<commit_message>
Update example test file WalkingRanges
Update reference test file for example WalkingRanges. After the style
infrastructure switch, the styles part is saved differently.
No semantic change to the styles part.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Ranges/WalkingRanges.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Ranges/WalkingRanges.xlsx
@@ -48,121 +48,82 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="7">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFA07A"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFADD8E6"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFA2A2D0"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFA8072"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF0000FF"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="6">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="6">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="7">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFA07A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFA8072"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFADD8E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA2A2D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000FF"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -467,29 +428,29 @@
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7">
-      <x:c r="C5" s="2" t="s">
+      <x:c r="C5" s="3" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D5" s="2" t="s">
+      <x:c r="D5" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F5" s="3" t="s">
+      <x:c r="F5" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G5" s="3" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
-      <x:c r="E6" s="4" t="s">
+      <x:c r="E6" s="2" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7">
-      <x:c r="E7" s="4" t="s">
+      <x:c r="E7" s="2" t="s">
         <x:v>8</x:v>
       </x:c>
     </x:row>
@@ -511,18 +472,18 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:4" s="1" customFormat="1"/>
-    <x:row r="2" spans="1:4" s="4" customFormat="1"/>
+    <x:row r="2" spans="1:4" s="2" customFormat="1"/>
     <x:row r="4" spans="1:4" s="5" customFormat="1"/>
-    <x:row r="5" spans="1:4" s="3" customFormat="1"/>
+    <x:row r="5" spans="1:4" s="4" customFormat="1"/>
     <x:row r="8" spans="1:4">
       <x:c r="B8" s="1"/>
       <x:c r="C8" s="1"/>
       <x:c r="D8" s="1"/>
     </x:row>
     <x:row r="9" spans="1:4">
-      <x:c r="B9" s="4"/>
-      <x:c r="C9" s="4"/>
-      <x:c r="D9" s="4"/>
+      <x:c r="B9" s="2"/>
+      <x:c r="C9" s="2"/>
+      <x:c r="D9" s="2"/>
     </x:row>
     <x:row r="11" spans="1:4">
       <x:c r="B11" s="5"/>
@@ -530,9 +491,9 @@
       <x:c r="D11" s="5"/>
     </x:row>
     <x:row r="12" spans="1:4">
-      <x:c r="B12" s="3"/>
-      <x:c r="C12" s="3"/>
-      <x:c r="D12" s="3"/>
+      <x:c r="B12" s="4"/>
+      <x:c r="C12" s="4"/>
+      <x:c r="D12" s="4"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -552,29 +513,29 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
-    <x:col min="2" max="2" width="9.140625" style="4" customWidth="1"/>
+    <x:col min="2" max="2" width="9.140625" style="2" customWidth="1"/>
     <x:col min="3" max="3" width="9.140625" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.140625" style="5" customWidth="1"/>
-    <x:col min="5" max="5" width="9.140625" style="3" customWidth="1"/>
+    <x:col min="5" max="5" width="9.140625" style="4" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2" spans="1:12">
       <x:c r="H2" s="1"/>
-      <x:c r="I2" s="4"/>
+      <x:c r="I2" s="2"/>
       <x:c r="K2" s="5"/>
-      <x:c r="L2" s="3"/>
+      <x:c r="L2" s="4"/>
     </x:row>
     <x:row r="3" spans="1:12">
       <x:c r="H3" s="1"/>
-      <x:c r="I3" s="4"/>
+      <x:c r="I3" s="2"/>
       <x:c r="K3" s="5"/>
-      <x:c r="L3" s="3"/>
+      <x:c r="L3" s="4"/>
     </x:row>
     <x:row r="4" spans="1:12">
       <x:c r="H4" s="1"/>
-      <x:c r="I4" s="4"/>
+      <x:c r="I4" s="2"/>
       <x:c r="K4" s="5"/>
-      <x:c r="L4" s="3"/>
+      <x:c r="L4" s="4"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>